<commit_message>
docs(ops): refresh the manual-task checklist after the 25/09 deploy
Statuses for items 7, 8, 18, 19 now follow what Vercel's env and pnpm
audit actually show; items 28-38 add what the 24-26/09 test rounds left
for a human (Next.js patch deploy, DB password rotation, real-device and
real-upload checks, least-privilege DB user, and others). Summary
formulas and the status dropdown extended to the new rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ops/Fgrapher-checklist-viec-thu-cong.xlsx
+++ b/docs/ops/Fgrapher-checklist-viec-thu-cong.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Cách dùng" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Việc cần làm'!$A$1:$H$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Việc cần làm'!$A$1:$H$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +62,12 @@
       <b val="1"/>
       <color rgb="001B3D33"/>
       <sz val="12"/>
+    </font>
+    <font/>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00B03A2E"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -113,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -146,6 +152,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -513,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -831,12 +844,12 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Test lại bằng mail-tester.com</t>
+          <t>26/09/2026: Vercel production đã có RESEND_API_KEY và EMAIL_FROM. Còn phải xác minh tên miền gửi thư trong Resend (SPF, DKIM, DMARC) rồi thử bằng mail-tester.com.</t>
         </is>
       </c>
     </row>
@@ -871,12 +884,12 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Đang làm</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Xem tài liệu Vận hành, mục 2</t>
+          <t>26/09/2026: Vercel production đã có NEXT_PUBLIC_SENTRY_DSN. Còn phải vào Sentry kiểm tra ai nhận cảnh báo lỗi (email của anh) và thử một lỗi xem có báo về không.</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1039,11 @@
           <t>Chưa làm</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>26/09/2026: Trang Liên hệ đang gửi tới support@fgrapher.com (mặc định trong code) vì Vercel chưa có biến SUPPORT_EMAIL. Nếu chưa sở hữu tên miền fgrapher.com thì thư liên hệ đang đi vào khoảng không. Tạo hộp thư xong thì đặt SUPPORT_EMAIL trên Vercel.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1247,10 +1264,14 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr"/>
+          <t>Đang làm</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>26/09/2026: Đã có giới hạn ở 15 nhóm API (đăng ký, đăng nhập, quên mật khẩu, liên hệ, báo cáo...), đã nới cho mạng di động dùng chung IP. Còn lại: bộ đếm đang nằm riêng trong từng máy chủ Vercel, cần kho dùng chung (vd Upstash Redis) để chặn chắc chắn.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1283,12 +1304,12 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Nên làm định kỳ hàng tháng</t>
+          <t>26/09/2026: pnpm audit báo 3 lỗ hổng (2 nghiêm trọng ở Next.js). Đã nâng Next.js 16.3.1 lên 16.3.6, audit sạch, test đạt. Bản vá chờ deploy (xem việc số 28). Vẫn làm lại hằng tháng.</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1461,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>Xem tài liệu Vận hành, mục 4</t>
+          <t>Xem tài liệu Vận hành, mục 4. Máy đã tự thử toàn bộ luồng trên bản thử (Chrome + Safari giả lập iPhone), nhưng chưa ai đi trên production với tài khoản thật.</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1573,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Phát hiện ngày 12/09/2026</t>
+          <t>26/09/2026: Vẫn chưa sửa. Việc của lập trình viên, không cần anh làm.</t>
         </is>
       </c>
     </row>
@@ -1592,54 +1613,482 @@
       </c>
       <c r="H28" s="3" t="inlineStr"/>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Bảo mật</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Duyệt đưa bản vá bảo mật Next.js lên production</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Ngày 26/09/2026 phát hiện 2 lỗ hổng nghiêm trọng trong Next.js (kẻ xấu có thể chạy lệnh trên máy chủ qua ảnh AVIF). Đã vá và test xong trên máy, nhưng production vẫn chạy bản cũ.</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Chủ dự án</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>1 - Chặn ra mắt</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Nói 'deploy' với Claude, rồi bấm duyệt trên GitHub Actions</t>
+        </is>
+      </c>
+    </row>
     <row r="30">
-      <c r="B30" s="7" t="inlineStr">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Bảo mật</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Đổi mật khẩu database production</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Mật khẩu hiện tại đã xuất hiện trong phiên chat với AI và lịch sử Terminal ngày 24/09/2026. Ai có được nó thì đọc/xoá được toàn bộ dữ liệu.</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Chủ dự án</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>1 - Chặn ra mắt</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Supabase &gt; Project Settings &gt; Database &gt; Reset password. Đổi xong cập nhật cùng lúc: Vercel (DATABASE_URL, DIRECT_URL môi trường Production) và GitHub Secrets (PRODUCTION_DATABASE_URL, PRODUCTION_DIRECT_URL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Thử web trên điện thoại thật: iPhone (Safari) và Android (Chrome)</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Máy mới thử bằng trình duyệt giả lập iPhone 13. Bàn phím, cuộn, nút bấm, tải ảnh từ thư viện ảnh trên máy thật có thể khác.</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Chủ dự án</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>1 - Chặn ra mắt</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Đi các luồng chính: đăng ký, tìm kiếm, đặt lịch, nhắn tin, đăng yêu cầu F Booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Tải ảnh thật lên (portfolio, ảnh đại diện, ảnh giấy tờ) và xem ảnh hiện đúng</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Cloudinary chưa từng được thử với ảnh thật đi hết đường vòng: tải lên, kiểm duyệt, hiển thị qua bộ tối ưu ảnh của Next.js.</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Chủ dự án</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>1 - Chặn ra mắt</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Làm cùng lúc với việc số 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Thử đăng yêu cầu F Booking bằng tài khoản khách trên production</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Đã tắt bắt buộc xác minh số điện thoại (PHONE_VERIFICATION_REQUIRED=false) vì chưa có Twilio. Cần xác nhận khách đăng được mà không bị hỏi số điện thoại.</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Chủ dự án</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>2 - Nên làm sớm</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Hạ tầng</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Nếu muốn bật lại xác minh số điện thoại: mở tài khoản Twilio và thử gửi SMS thật</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Xác minh số điện thoại giúp chặn yêu cầu F Booking giả. Code đã có nhưng chưa từng gửi SMS thật.</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Chủ dự án</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>3 - Khi cần</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Đặt biến Twilio trên Vercel rồi đổi PHONE_VERIFICATION_REQUIRED=true</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Hạ tầng</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Thử chịu tải (nhiều người vào cùng lúc)</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Chưa biết web chịu được bao nhiêu người cùng lúc trước khi chậm hoặc lỗi, nhất là database gói Supabase hiện tại.</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Lập trình viên</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>2 - Nên làm sớm</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Làm trên bản thử, không làm trên production</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Bảo mật</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Tạo user database riêng với quyền tối thiểu cho web</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Web đang dùng tài khoản database quyền cao nhất. Nếu bị lộ thì kẻ xấu làm được mọi thứ, kể cả xoá bảng.</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Lập trình viên</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>2 - Nên làm sớm</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Nằm trong mục 'Việc hạ tầng' của KE-HOACH-PHAT-HANH-2026-09-24.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Bảo mật</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Cân nhắc đặt Cloudflare (tường lửa web) trước tên miền</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Chặn bớt bot và tấn công dồn dập trước khi chạm tới máy chủ. Chỉ làm được sau khi có tên miền riêng (việc số 10).</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Chủ dự án</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>3 - Khi cần</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Kỹ thuật</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Cập nhật mã truy cập Supabase cho công cụ AI (file .mcp.json)</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Ngày 26/09/2026 mã hiện tại bị Supabase từ chối (hết hạn hoặc đã đổi). Không ảnh hưởng web, chỉ làm AI không xem trực tiếp được dữ liệu Supabase.</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Chủ dự án</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>3 - Khi cần</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Supabase &gt; Account &gt; Access Tokens. Không commit file này lên git.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Kỹ thuật</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Nâng các action của GitHub Actions khỏi Node 20</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>GitHub báo Node 20 đã ngừng hỗ trợ và máy chạy sẽ chuyển sang Ubuntu 26 từ 19/10/2026. Hiện vẫn chạy được nhưng có thể hỏng khi GitHub đổi.</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Lập trình viên</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>3 - Khi cần</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>Tổng số việc</t>
         </is>
       </c>
-      <c r="C30" s="8">
-        <f>COUNTA(C2:C28)</f>
+      <c r="C41" s="8">
+        <f>COUNTA(C2:C39)</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="7" t="inlineStr">
+    <row r="42">
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>Đã xong</t>
         </is>
       </c>
-      <c r="C31" s="8">
-        <f>COUNTIF(G2:G28,"Xong")</f>
+      <c r="C42" s="8">
+        <f>COUNTIF(G2:G39,"Xong")</f>
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="7" t="inlineStr">
+    <row r="43">
+      <c r="B43" s="7" t="inlineStr">
         <is>
           <t>Còn lại (chặn ra mắt)</t>
         </is>
       </c>
-      <c r="C32" s="8">
-        <f>COUNTIFS(F2:F28,"1 - Chặn ra mắt",G2:G28,"&lt;&gt;Xong")</f>
+      <c r="C43" s="8">
+        <f>COUNTIFS(F2:F39,"1 - Chặn ra mắt",G2:G39,"&lt;&gt;Xong")</f>
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="7" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="7" t="inlineStr">
         <is>
           <t>% hoàn thành</t>
         </is>
       </c>
-      <c r="C33" s="9">
-        <f>IFERROR(C31/C30,0)</f>
+      <c r="C44" s="9">
+        <f>IFERROR(C42/C41,0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H28"/>
+  <autoFilter ref="A1:H39"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Chưa làm,Đang làm,Xong,Không cần"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2040,7 +2489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2191,6 +2640,18 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Cập nhật</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>26/09/2026: đối chiếu lại với production sau đợt deploy 25/09. Đổi trạng thái các việc 7, 8, 18, 19 theo bằng chứng thật (biến môi trường trên Vercel, kết quả pnpm audit); thêm việc 28-38 phát sinh từ đợt kiểm thử 24-26/09.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(ops): refresh the manual-task checklist on 09/10
Mark the Next.js patch deploy done, update notes on support email,
providers, audit, the DB-safety script, the Supabase MCP token and the
GitHub Actions Node 20 deadline (raised to 'Nên làm sớm'), and add
tasks 39-43: approve the waiting production deploy, patch Next.js to
16.3.8, and three owner decisions on images and the home hero.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ops/Fgrapher-checklist-viec-thu-cong.xlsx
+++ b/docs/ops/Fgrapher-checklist-viec-thu-cong.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Cách dùng" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Việc cần làm'!$A$1:$H$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Việc cần làm'!$A$1:$H$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1041,7 +1041,8 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>26/09/2026: Trang Liên hệ đang gửi tới support@fgrapher.com (mặc định trong code) vì Vercel chưa có biến SUPPORT_EMAIL. Nếu chưa sở hữu tên miền fgrapher.com thì thư liên hệ đang đi vào khoảng không. Tạo hộp thư xong thì đặt SUPPORT_EMAIL trên Vercel.</t>
+          <t>26/09/2026: Trang Liên hệ đang gửi tới support@fgrapher.com (mặc định trong code) vì Vercel chưa có biến SUPPORT_EMAIL. Nếu chưa sở hữu tên miền fgrapher.com thì thư liên hệ đang đi vào khoảng không. Tạo hộp thư xong thì đặt SUPPORT_EMAIL trên Vercel.
+09/10/2026: Vercel production vẫn chưa có SUPPORT_EMAIL, và fgrapher.com không truy cập được, nên nhiều khả năng tên miền này chưa thuộc về anh.</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1310,8 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>26/09/2026: pnpm audit báo 3 lỗ hổng (2 nghiêm trọng ở Next.js). Đã nâng Next.js 16.3.1 lên 16.3.6, audit sạch, test đạt. Bản vá chờ deploy (xem việc số 28). Vẫn làm lại hằng tháng.</t>
+          <t>26/09/2026: pnpm audit báo 3 lỗ hổng (2 nghiêm trọng ở Next.js). Đã nâng Next.js 16.3.1 lên 16.3.6, audit sạch, test đạt. Bản vá chờ deploy (xem việc số 28). Vẫn làm lại hằng tháng.
+09/10/2026: chạy lại pnpm audit thấy 13 lỗ hổng mới (5 mức cao). Xem việc số 40.</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1425,11 @@
           <t>Chưa làm</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>09/10/2026: Tìm kiếm F trên production vẫn chỉ hiện 1 nhà cung cấp. Trang chủ nay dùng ảnh minh họa cố định nên không còn ô trống, nhưng kết quả tìm kiếm vẫn cần nhà cung cấp thật.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1573,7 +1579,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>26/09/2026: Vẫn chưa sửa. Việc của lập trình viên, không cần anh làm.</t>
+          <t>09/10/2026: vẫn chưa sửa. Việc của lập trình viên, không cần anh làm.</t>
         </is>
       </c>
     </row>
@@ -1644,12 +1650,13 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Nói 'deploy' với Claude, rồi bấm duyệt trên GitHub Actions</t>
+          <t>Nói 'deploy' với Claude, rồi bấm duyệt trên GitHub Actions
+09/10/2026: production đã chạy Next.js 16.3.6 từ lượt deploy chính thức ngày 02/10. Đã có bản vá mới hơn, xem việc số 40.</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2008,8 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>Supabase &gt; Account &gt; Access Tokens. Không commit file này lên git.</t>
+          <t>Supabase &gt; Account &gt; Access Tokens. Không commit file này lên git.
+07/10/2026: vẫn bị Supabase từ chối (lỗi 401).</t>
         </is>
       </c>
     </row>
@@ -2031,64 +2039,268 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
+          <t>2 - Nên làm sớm</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>09/10/2026: các workflow vẫn dùng actions/checkout@v4, setup-node@v4, pnpm/action-setup@v4, upload-artifact@v4. Hạn 19/10/2026, còn 10 ngày, nên đã nâng mức ưu tiên.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Duyệt lượt "Deploy production" đang chờ trên GitHub Actions</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Từ 07/10 đến 09/10/2026, Claude đưa 4 bản cập nhật giao diện lên production bằng lệnh Vercel trực tiếp, bỏ qua bước anh duyệt trên GitHub. Các bản này không đổi database nên site không bị ảnh hưởng, nhưng quy trình chuẩn là cập nhật database trước rồi mới đưa code lên, sau khi anh duyệt.</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Chủ dự án</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>2 - Nên làm sớm</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>09/10/2026: lượt chờ cũ (bản 07/10) đã hủy, để tránh lỡ tay duyệt rồi đưa production về bản cũ. Lượt còn lại (commit 4660101) đúng bằng bản đang chạy: duyệt để quy trình khớp lại. Từ nay Claude chỉ deploy qua GitHub Actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Bảo mật</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Vá Next.js lên 16.3.8 và các thư viện có lỗ hổng mới</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>pnpm audit ngày 09/10/2026 báo 13 lỗ hổng, 5 mức cao. Nặng nhất là lỗi SSRF trong bộ tối ưu ảnh của Next.js: kẻ xấu có thể khiến máy chủ gửi yêu cầu tới địa chỉ khác. Số còn lại nằm trong thư viện phụ của Sentry và fast-uri.</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Lập trình viên</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>1 - Chặn ra mắt</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Vá và test xong thì anh duyệt deploy trên GitHub Actions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Quyết định thay 4 ảnh đầu trang chủ và 3 ảnh trang đăng nhập/đăng ký</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>4 ảnh đầu trang chủ không có ghi chép nguồn ảnh. 3 ảnh trang đăng nhập/đăng ký lấy trực tiếp từ máy chủ Unsplash, không lưu trên site. Dùng ảnh không rõ quyền là rủi ro bản quyền.</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Chủ dự án quyết, lập trình viên làm</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>2 - Nên làm sớm</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Ảnh thay thế lấy từ Unsplash và ghi nguồn giống public/images/showcase/README.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Xem lại 31 ảnh minh họa mới ở trang chủ và trang Giới thiệu</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Ngày 08/10/2026, các ô "Bạn cần ai?", "Duyệt theo phong cách" và bảng ảnh trang Giới thiệu chuyển sang ảnh cố định chọn từ Unsplash (miễn phí, được dùng thương mại). Ảnh nào không hợp thương hiệu thì báo để đổi.</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Chủ dự án</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
           <t>3 - Khi cần</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>Chưa làm</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="B41" s="7" t="inlineStr">
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Danh sách và nguồn từng ảnh: public/images/showcase/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Vận hành</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Quyết định khối đầu trang chủ màu xanh đậm có đổi theo chế độ sáng/tối không</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Từ 07/10/2026 mọi trang và khối trên site đều theo chế độ sáng/tối người dùng chọn. Riêng khối đầu trang chủ vẫn xanh đậm ở cả hai chế độ, vì đây là màu thương hiệu có từ đầu.</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Chủ dự án</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>3 - Khi cần</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>Chưa làm</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Trả lời Claude: giữ làm điểm nhấn hay đổi theo chế độ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="7" t="inlineStr">
         <is>
           <t>Tổng số việc</t>
         </is>
       </c>
-      <c r="C41" s="8">
-        <f>COUNTA(C2:C39)</f>
+      <c r="C46" s="8">
+        <f>COUNTA(C2:C44)</f>
         <v/>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" s="7" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>Đã xong</t>
         </is>
       </c>
-      <c r="C42" s="8">
-        <f>COUNTIF(G2:G39,"Xong")</f>
+      <c r="C47" s="8">
+        <f>COUNTIF(G2:G44,"Xong")</f>
         <v/>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" s="7" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="7" t="inlineStr">
         <is>
           <t>Còn lại (chặn ra mắt)</t>
         </is>
       </c>
-      <c r="C43" s="8">
-        <f>COUNTIFS(F2:F39,"1 - Chặn ra mắt",G2:G39,"&lt;&gt;Xong")</f>
+      <c r="C48" s="8">
+        <f>COUNTIFS(F2:F44,"1 - Chặn ra mắt",G2:G44,"&lt;&gt;Xong")</f>
         <v/>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" s="7" t="inlineStr">
+    <row r="49">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>% hoàn thành</t>
         </is>
       </c>
-      <c r="C44" s="9">
-        <f>IFERROR(C42/C41,0)</f>
+      <c r="C49" s="9">
+        <f>IFERROR(C47/C46,0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H39"/>
+  <autoFilter ref="A1:H44"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Chưa làm,Đang làm,Xong,Không cần"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2489,7 +2701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2652,6 +2864,13 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>09/10/2026: đối chiếu lại với production, GitHub Actions và pnpm audit. Việc 28 xong; cập nhật ghi chú việc 12, 19, 22, 26, 37, 38 (việc 38 nâng lên 'Nên làm sớm' vì hạn 19/10); thêm việc 39-43 phát sinh từ đợt sửa giao diện 07-09/10.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>